<commit_message>
fix: adiciona esforço horas nos projetos AASP_AP, PROFARMA, AASP_CNJ
Dados extraídos das planilhas de gestão (GEST .xlsx) e PLA:
- AASP_AP: 362h realizadas (Fases 1-4; GEST-AASPAP01 aba Acompanhamento)
- PROFARMA: 5.789h estimadas (PLA-PROFARMA01-001 §4 orçamento por papel)
- AASP_CNJ: 624h realizadas (GEST-AASPCNJ01 aba Medição, Fases 1-6)
- FRUKI: usa Story Points (GEST-FRUKI), sem total em horas disponível

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011KXfcc9u9SbkrrmomU4zNq
</commit_message>
<xml_diff>
--- a/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
+++ b/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
@@ -15695,7 +15695,9 @@
           <t>Construção</t>
         </is>
       </c>
-      <c r="F6" s="71" t="n"/>
+      <c r="F6" s="71" t="n">
+        <v>362</v>
+      </c>
       <c r="G6" s="71" t="n">
         <v>4</v>
       </c>
@@ -15755,7 +15757,9 @@
           <t>Concluído</t>
         </is>
       </c>
-      <c r="F7" s="71" t="n"/>
+      <c r="F7" s="71" t="n">
+        <v>5789</v>
+      </c>
       <c r="G7" s="71" t="n">
         <v>9</v>
       </c>
@@ -15817,7 +15821,9 @@
           <t>Construção</t>
         </is>
       </c>
-      <c r="F8" s="71" t="n"/>
+      <c r="F8" s="71" t="n">
+        <v>624</v>
+      </c>
       <c r="G8" s="71" t="n">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
pré-avaliação: atualiza esforço FRUKI para 2.058h realizadas
Substitui esforco=None por esforco=2058 no script _fill_pre_avaliacao.py,
com base em MED-FRUKI01-001 v1.1 (Pacote 1: ~847h + Pacote Final 24: ~1.211h).
Regenera PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx com o valor correto.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
+++ b/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
@@ -15633,7 +15633,9 @@
           <t>Concluído</t>
         </is>
       </c>
-      <c r="F5" s="71" t="n"/>
+      <c r="F5" s="71" t="n">
+        <v>2058</v>
+      </c>
       <c r="G5" s="71" t="n">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
pré-avaliação: preenche Sprint ou Fase no PLANO para todos os projetos
Adiciona campo sprint_ou_fase em cada projeto e escreve na col D do PLANO:
- FTFRUKI: Concluído
- AASP_AP: Fase 5 — Implantação (ATA-AASPAP01-005)
- PROFARMA: Concluído
- AASP_CNJ: Fase 7 — Homologação / Encerramento (00_INDICE-AASPCNJ01)

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
+++ b/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
@@ -17582,7 +17582,11 @@
         <f>iferror(vlookup($A17,InstanciasSelecionadas,3,false),"-")</f>
         <v/>
       </c>
-      <c r="D17" s="92" t="n"/>
+      <c r="D17" s="92" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
       <c r="E17" s="92">
         <f>iferror(vlookup($A17,InstanciasSelecionadas,4,false),"-")</f>
         <v/>
@@ -17602,7 +17606,11 @@
         <f>iferror(vlookup($A18,InstanciasSelecionadas,3,false),"-")</f>
         <v/>
       </c>
-      <c r="D18" s="92" t="n"/>
+      <c r="D18" s="92" t="inlineStr">
+        <is>
+          <t>Fase 5 — Implantação</t>
+        </is>
+      </c>
       <c r="E18" s="92">
         <f>iferror(vlookup($A18,InstanciasSelecionadas,4,false),"-")</f>
         <v/>
@@ -17622,7 +17630,11 @@
         <f>iferror(vlookup($A19,InstanciasSelecionadas,3,false),"-")</f>
         <v/>
       </c>
-      <c r="D19" s="92" t="n"/>
+      <c r="D19" s="92" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
       <c r="E19" s="92">
         <f>iferror(vlookup($A19,InstanciasSelecionadas,4,false),"-")</f>
         <v/>
@@ -17642,7 +17654,11 @@
         <f>iferror(vlookup($A20,InstanciasSelecionadas,3,false),"-")</f>
         <v/>
       </c>
-      <c r="D20" s="92" t="n"/>
+      <c r="D20" s="92" t="inlineStr">
+        <is>
+          <t>Fase 7 — Homologação / Encerramento</t>
+        </is>
+      </c>
       <c r="E20" s="92">
         <f>iferror(vlookup($A20,InstanciasSelecionadas,4,false),"-")</f>
         <v/>

</xml_diff>

<commit_message>
pré-avaliação: corrige equipe AASP_AP e AASP_CNJ com todos os membros
AASP_AP: adiciona Mateus Veloso e Caroline Sousa (presentes ATA Fase 4);
envolvidos 4→5. AASP_CNJ: substitui nomes incorretos (Levi Santos, Jonatan
Silva, David Buena) pelos nomes do TAP (Mateus Veloso, Lucas Batista,
Caroline Sousa, Jonathan Barbosa GQA); envolvidos 6→7.

Co-Authored-By: Claude Sonnet <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
+++ b/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
@@ -15701,7 +15701,7 @@
         <v>362</v>
       </c>
       <c r="G6" s="71" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="71" t="inlineStr">
         <is>
@@ -15827,7 +15827,7 @@
         <v>624</v>
       </c>
       <c r="G8" s="71" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H8" s="71" t="inlineStr">
         <is>
@@ -18556,32 +18556,32 @@
     <row r="12">
       <c r="A12" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B12" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>Mateus Veloso</t>
         </is>
       </c>
       <c r="C12" s="267" t="inlineStr">
         <is>
-          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
+          <t>AASP — Andamento Processuais</t>
         </is>
       </c>
       <c r="D12" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projeto / Account Manager</t>
+          <t>Desenvolvedor (Suporte)</t>
         </is>
       </c>
       <c r="E12" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projetos</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F12" s="267" t="inlineStr">
         <is>
-          <t>Wilson Yamada</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G12" s="268" t="n"/>
@@ -18595,30 +18595,34 @@
     <row r="13">
       <c r="A13" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B13" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Caroline Sousa</t>
         </is>
       </c>
       <c r="C13" s="267" t="inlineStr">
         <is>
-          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
+          <t>AASP — Andamento Processuais</t>
         </is>
       </c>
       <c r="D13" s="267" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Analista de QA</t>
         </is>
       </c>
       <c r="E13" s="267" t="inlineStr">
         <is>
-          <t>CEO / Founder</t>
-        </is>
-      </c>
-      <c r="F13" s="267" t="inlineStr"/>
+          <t>Analista de QA</t>
+        </is>
+      </c>
+      <c r="F13" s="267" t="inlineStr">
+        <is>
+          <t>Abraão Oliveira</t>
+        </is>
+      </c>
       <c r="G13" s="268" t="n"/>
       <c r="H13" s="114" t="n"/>
       <c r="I13" s="115">
@@ -18630,12 +18634,12 @@
     <row r="14">
       <c r="A14" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B14" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="C14" s="267" t="inlineStr">
@@ -18645,17 +18649,17 @@
       </c>
       <c r="D14" s="267" t="inlineStr">
         <is>
-          <t>Dev Principal / Arquiteto da solução</t>
+          <t>Gerente de Projeto / Account Manager</t>
         </is>
       </c>
       <c r="E14" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>Gerente de Projetos</t>
         </is>
       </c>
       <c r="F14" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Wilson Yamada</t>
         </is>
       </c>
       <c r="G14" s="268" t="n"/>
@@ -18666,12 +18670,12 @@
     <row r="15">
       <c r="A15" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B15" s="267" t="inlineStr">
         <is>
-          <t>Gustavo Mathias</t>
+          <t>Tiago Barbosa Nascimento</t>
         </is>
       </c>
       <c r="C15" s="267" t="inlineStr">
@@ -18681,19 +18685,15 @@
       </c>
       <c r="D15" s="267" t="inlineStr">
         <is>
-          <t>Dev Backend</t>
+          <t>Tech Lead</t>
         </is>
       </c>
       <c r="E15" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior</t>
-        </is>
-      </c>
-      <c r="F15" s="267" t="inlineStr">
-        <is>
-          <t>Erick Coelho</t>
-        </is>
-      </c>
+          <t>CEO / Founder</t>
+        </is>
+      </c>
+      <c r="F15" s="267" t="inlineStr"/>
       <c r="G15" s="268" t="n"/>
       <c r="H15" s="268" t="n"/>
       <c r="I15" s="109" t="n"/>
@@ -18707,7 +18707,7 @@
       </c>
       <c r="B16" s="267" t="inlineStr">
         <is>
-          <t>Renan Kiyoshi</t>
+          <t>Erick Coelho</t>
         </is>
       </c>
       <c r="C16" s="267" t="inlineStr">
@@ -18717,17 +18717,17 @@
       </c>
       <c r="D16" s="267" t="inlineStr">
         <is>
-          <t>Dev Backend</t>
+          <t>Dev Principal / Arquiteto da solução</t>
         </is>
       </c>
       <c r="E16" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior</t>
+          <t>Arquiteto de Software</t>
         </is>
       </c>
       <c r="F16" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Tiago Barbosa Nascimento</t>
         </is>
       </c>
       <c r="G16" s="268" t="n"/>
@@ -18743,7 +18743,7 @@
       </c>
       <c r="B17" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Gustavo Mathias</t>
         </is>
       </c>
       <c r="C17" s="267" t="inlineStr">
@@ -18758,12 +18758,12 @@
       </c>
       <c r="E17" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>Desenvolvedor Sênior</t>
         </is>
       </c>
       <c r="F17" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Erick Coelho</t>
         </is>
       </c>
       <c r="G17" s="268" t="n"/>
@@ -18779,7 +18779,7 @@
       </c>
       <c r="B18" s="267" t="inlineStr">
         <is>
-          <t>João Cruz</t>
+          <t>Renan Kiyoshi</t>
         </is>
       </c>
       <c r="C18" s="267" t="inlineStr">
@@ -18794,7 +18794,7 @@
       </c>
       <c r="E18" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Desenvolvedor Sênior</t>
         </is>
       </c>
       <c r="F18" s="267" t="inlineStr">
@@ -18815,7 +18815,7 @@
       </c>
       <c r="B19" s="267" t="inlineStr">
         <is>
-          <t>David Buena</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="C19" s="267" t="inlineStr">
@@ -18825,17 +18825,17 @@
       </c>
       <c r="D19" s="267" t="inlineStr">
         <is>
-          <t>Infra / DevOps</t>
+          <t>Dev Backend</t>
         </is>
       </c>
       <c r="E19" s="267" t="inlineStr">
         <is>
-          <t>Engenheiro DevOps</t>
+          <t>Arquiteto de Software</t>
         </is>
       </c>
       <c r="F19" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Tiago Barbosa Nascimento</t>
         </is>
       </c>
       <c r="G19" s="268" t="n"/>
@@ -18851,7 +18851,7 @@
       </c>
       <c r="B20" s="267" t="inlineStr">
         <is>
-          <t>Lucas Batista</t>
+          <t>João Cruz</t>
         </is>
       </c>
       <c r="C20" s="267" t="inlineStr">
@@ -18861,17 +18861,17 @@
       </c>
       <c r="D20" s="267" t="inlineStr">
         <is>
-          <t>QA / Testes Automatizados</t>
+          <t>Dev Backend</t>
         </is>
       </c>
       <c r="E20" s="267" t="inlineStr">
         <is>
-          <t>Analista de QA</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F20" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>Erick Coelho</t>
         </is>
       </c>
       <c r="G20" s="268" t="n"/>
@@ -18882,32 +18882,32 @@
     <row r="21">
       <c r="A21" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B21" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>David Buena</t>
         </is>
       </c>
       <c r="C21" s="267" t="inlineStr">
         <is>
-          <t>AASP — CNJ Integração</t>
+          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
         </is>
       </c>
       <c r="D21" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projeto / Tech Lead</t>
+          <t>Infra / DevOps</t>
         </is>
       </c>
       <c r="E21" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projetos</t>
+          <t>Engenheiro DevOps</t>
         </is>
       </c>
       <c r="F21" s="267" t="inlineStr">
         <is>
-          <t>Wilson Yamada</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G21" s="268" t="n"/>
@@ -18918,27 +18918,27 @@
     <row r="22">
       <c r="A22" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B22" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Lucas Batista</t>
         </is>
       </c>
       <c r="C22" s="267" t="inlineStr">
         <is>
-          <t>AASP — CNJ Integração</t>
+          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
         </is>
       </c>
       <c r="D22" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>QA / Testes Automatizados</t>
         </is>
       </c>
       <c r="E22" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>Analista de QA</t>
         </is>
       </c>
       <c r="F22" s="267" t="inlineStr">
@@ -18954,12 +18954,12 @@
     <row r="23">
       <c r="A23" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B23" s="267" t="inlineStr">
         <is>
-          <t>Raony Chagas</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="C23" s="267" t="inlineStr">
@@ -18969,17 +18969,17 @@
       </c>
       <c r="D23" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior (Principal)</t>
+          <t>Gerente de Projeto</t>
         </is>
       </c>
       <c r="E23" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior</t>
+          <t>Gerente de Projetos</t>
         </is>
       </c>
       <c r="F23" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Wilson Yamada</t>
         </is>
       </c>
       <c r="G23" s="268" t="n"/>
@@ -18990,12 +18990,12 @@
     <row r="24">
       <c r="A24" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B24" s="267" t="inlineStr">
         <is>
-          <t>Levi Santos</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="C24" s="267" t="inlineStr">
@@ -19005,17 +19005,17 @@
       </c>
       <c r="D24" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor (Suporte)</t>
+          <t>Tech Lead / DevOps / Arquiteto</t>
         </is>
       </c>
       <c r="E24" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Arquiteto de Software</t>
         </is>
       </c>
       <c r="F24" s="267" t="inlineStr">
         <is>
-          <t>Raony Chagas</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G24" s="268" t="n"/>
@@ -19031,7 +19031,7 @@
       </c>
       <c r="B25" s="267" t="inlineStr">
         <is>
-          <t>Jonatan Silva</t>
+          <t>Raony Chagas</t>
         </is>
       </c>
       <c r="C25" s="267" t="inlineStr">
@@ -19041,17 +19041,17 @@
       </c>
       <c r="D25" s="267" t="inlineStr">
         <is>
-          <t>Analista de Testes</t>
+          <t>Desenvolvedor Sênior (Principal)</t>
         </is>
       </c>
       <c r="E25" s="267" t="inlineStr">
         <is>
-          <t>Analista de QA</t>
+          <t>Desenvolvedor Sênior</t>
         </is>
       </c>
       <c r="F25" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G25" s="268" t="n"/>
@@ -19067,7 +19067,7 @@
       </c>
       <c r="B26" s="267" t="inlineStr">
         <is>
-          <t>David Buena</t>
+          <t>Mateus Veloso</t>
         </is>
       </c>
       <c r="C26" s="267" t="inlineStr">
@@ -19077,12 +19077,12 @@
       </c>
       <c r="D26" s="267" t="inlineStr">
         <is>
-          <t>Infraestrutura / DevOps</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="E26" s="267" t="inlineStr">
         <is>
-          <t>Engenheiro DevOps</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F26" s="267" t="inlineStr">
@@ -19096,36 +19096,108 @@
       <c r="J26" s="268" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="267" t="n"/>
-      <c r="B27" s="267" t="n"/>
-      <c r="C27" s="267" t="n"/>
-      <c r="D27" s="267" t="n"/>
-      <c r="E27" s="267" t="n"/>
-      <c r="F27" s="267" t="n"/>
+      <c r="A27" s="267" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B27" s="267" t="inlineStr">
+        <is>
+          <t>Lucas Batista</t>
+        </is>
+      </c>
+      <c r="C27" s="267" t="inlineStr">
+        <is>
+          <t>AASP — CNJ Integração</t>
+        </is>
+      </c>
+      <c r="D27" s="267" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="E27" s="267" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="F27" s="267" t="inlineStr">
+        <is>
+          <t>Cézar Hiraki Velázquez</t>
+        </is>
+      </c>
       <c r="G27" s="268" t="n"/>
       <c r="H27" s="268" t="n"/>
       <c r="I27" s="109" t="n"/>
       <c r="J27" s="268" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="267" t="n"/>
-      <c r="B28" s="267" t="n"/>
-      <c r="C28" s="267" t="n"/>
-      <c r="D28" s="267" t="n"/>
-      <c r="E28" s="267" t="n"/>
-      <c r="F28" s="267" t="n"/>
+      <c r="A28" s="267" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B28" s="267" t="inlineStr">
+        <is>
+          <t>Caroline Sousa</t>
+        </is>
+      </c>
+      <c r="C28" s="267" t="inlineStr">
+        <is>
+          <t>AASP — CNJ Integração</t>
+        </is>
+      </c>
+      <c r="D28" s="267" t="inlineStr">
+        <is>
+          <t>Analista de QA</t>
+        </is>
+      </c>
+      <c r="E28" s="267" t="inlineStr">
+        <is>
+          <t>Analista de QA</t>
+        </is>
+      </c>
+      <c r="F28" s="267" t="inlineStr">
+        <is>
+          <t>Abraão Oliveira</t>
+        </is>
+      </c>
       <c r="G28" s="268" t="n"/>
       <c r="H28" s="268" t="n"/>
       <c r="I28" s="109" t="n"/>
       <c r="J28" s="268" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="267" t="n"/>
-      <c r="B29" s="267" t="n"/>
-      <c r="C29" s="267" t="n"/>
-      <c r="D29" s="267" t="n"/>
-      <c r="E29" s="267" t="n"/>
-      <c r="F29" s="267" t="n"/>
+      <c r="A29" s="267" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B29" s="267" t="inlineStr">
+        <is>
+          <t>Jonathan Barbosa</t>
+        </is>
+      </c>
+      <c r="C29" s="267" t="inlineStr">
+        <is>
+          <t>AASP — CNJ Integração</t>
+        </is>
+      </c>
+      <c r="D29" s="267" t="inlineStr">
+        <is>
+          <t>Auditor GQA (independente)</t>
+        </is>
+      </c>
+      <c r="E29" s="267" t="inlineStr">
+        <is>
+          <t>Analista de Qualidade</t>
+        </is>
+      </c>
+      <c r="F29" s="267" t="inlineStr">
+        <is>
+          <t>Abraão Oliveira</t>
+        </is>
+      </c>
       <c r="G29" s="268" t="n"/>
       <c r="H29" s="268" t="n"/>
       <c r="I29" s="109" t="n"/>

</xml_diff>

<commit_message>
Reconciliação de documentos cadastro-clientes
</commit_message>
<xml_diff>
--- a/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
+++ b/mps-nivel-c/_interno/PlanilhaAvaliacao_TIMEWARE_SW_C_PREENCHIDA.xlsx
@@ -18163,7 +18163,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J500"/>
+  <dimension ref="A1:J497"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="13.75" customWidth="1" style="384" min="1" max="1"/>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B15" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="C15" s="267" t="inlineStr">
@@ -18685,15 +18685,19 @@
       </c>
       <c r="D15" s="267" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Tech Lead / DevOps / Arquiteto</t>
         </is>
       </c>
       <c r="E15" s="267" t="inlineStr">
         <is>
-          <t>CEO / Founder</t>
-        </is>
-      </c>
-      <c r="F15" s="267" t="inlineStr"/>
+          <t>Arquiteto de Software</t>
+        </is>
+      </c>
+      <c r="F15" s="267" t="inlineStr">
+        <is>
+          <t>Abraão Oliveira</t>
+        </is>
+      </c>
       <c r="G15" s="268" t="n"/>
       <c r="H15" s="268" t="n"/>
       <c r="I15" s="109" t="n"/>
@@ -18707,7 +18711,7 @@
       </c>
       <c r="B16" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Mateus Veloso</t>
         </is>
       </c>
       <c r="C16" s="267" t="inlineStr">
@@ -18717,17 +18721,17 @@
       </c>
       <c r="D16" s="267" t="inlineStr">
         <is>
-          <t>Dev Principal / Arquiteto da solução</t>
+          <t>Dev Backend</t>
         </is>
       </c>
       <c r="E16" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F16" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G16" s="268" t="n"/>
@@ -18743,7 +18747,7 @@
       </c>
       <c r="B17" s="267" t="inlineStr">
         <is>
-          <t>Gustavo Mathias</t>
+          <t>Raony Chagas</t>
         </is>
       </c>
       <c r="C17" s="267" t="inlineStr">
@@ -18763,7 +18767,7 @@
       </c>
       <c r="F17" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G17" s="268" t="n"/>
@@ -18779,7 +18783,7 @@
       </c>
       <c r="B18" s="267" t="inlineStr">
         <is>
-          <t>Renan Kiyoshi</t>
+          <t>Lucas Batista</t>
         </is>
       </c>
       <c r="C18" s="267" t="inlineStr">
@@ -18794,12 +18798,12 @@
       </c>
       <c r="E18" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F18" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G18" s="268" t="n"/>
@@ -18815,7 +18819,7 @@
       </c>
       <c r="B19" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Caroline Sousa</t>
         </is>
       </c>
       <c r="C19" s="267" t="inlineStr">
@@ -18825,17 +18829,17 @@
       </c>
       <c r="D19" s="267" t="inlineStr">
         <is>
-          <t>Dev Backend</t>
+          <t>QA / Testes Automatizados</t>
         </is>
       </c>
       <c r="E19" s="267" t="inlineStr">
         <is>
-          <t>Arquiteto de Software</t>
+          <t>Analista de QA</t>
         </is>
       </c>
       <c r="F19" s="267" t="inlineStr">
         <is>
-          <t>Tiago Barbosa Nascimento</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G19" s="268" t="n"/>
@@ -18846,32 +18850,32 @@
     <row r="20">
       <c r="A20" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B20" s="267" t="inlineStr">
         <is>
-          <t>João Cruz</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="C20" s="267" t="inlineStr">
         <is>
-          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
+          <t>AASP — CNJ Integração</t>
         </is>
       </c>
       <c r="D20" s="267" t="inlineStr">
         <is>
-          <t>Dev Backend</t>
+          <t>Gerente de Projeto</t>
         </is>
       </c>
       <c r="E20" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Gerente de Projetos</t>
         </is>
       </c>
       <c r="F20" s="267" t="inlineStr">
         <is>
-          <t>Erick Coelho</t>
+          <t>Wilson Yamada</t>
         </is>
       </c>
       <c r="G20" s="268" t="n"/>
@@ -18882,32 +18886,32 @@
     <row r="21">
       <c r="A21" s="267" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="B21" s="267" t="inlineStr">
         <is>
-          <t>David Buena</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="C21" s="267" t="inlineStr">
         <is>
-          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
+          <t>AASP — CNJ Integração</t>
         </is>
       </c>
       <c r="D21" s="267" t="inlineStr">
         <is>
-          <t>Infra / DevOps</t>
+          <t>Tech Lead / DevOps / Arquiteto</t>
         </is>
       </c>
       <c r="E21" s="267" t="inlineStr">
         <is>
-          <t>Engenheiro DevOps</t>
+          <t>Arquiteto de Software</t>
         </is>
       </c>
       <c r="F21" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G21" s="268" t="n"/>
@@ -18923,27 +18927,27 @@
       </c>
       <c r="B22" s="267" t="inlineStr">
         <is>
-          <t>Lucas Batista</t>
+          <t>Raony Chagas</t>
         </is>
       </c>
       <c r="C22" s="267" t="inlineStr">
         <is>
-          <t>PROFARMA / D1000 — Cadastro de Clientes</t>
+          <t>AASP — CNJ Integração</t>
         </is>
       </c>
       <c r="D22" s="267" t="inlineStr">
         <is>
-          <t>QA / Testes Automatizados</t>
+          <t>Desenvolvedor Sênior (Principal)</t>
         </is>
       </c>
       <c r="E22" s="267" t="inlineStr">
         <is>
-          <t>Analista de QA</t>
+          <t>Desenvolvedor Sênior</t>
         </is>
       </c>
       <c r="F22" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G22" s="268" t="n"/>
@@ -18954,12 +18958,12 @@
     <row r="23">
       <c r="A23" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B23" s="267" t="inlineStr">
         <is>
-          <t>Abraão Oliveira</t>
+          <t>Mateus Veloso</t>
         </is>
       </c>
       <c r="C23" s="267" t="inlineStr">
@@ -18969,17 +18973,17 @@
       </c>
       <c r="D23" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projeto</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="E23" s="267" t="inlineStr">
         <is>
-          <t>Gerente de Projetos</t>
+          <t>Desenvolvedor</t>
         </is>
       </c>
       <c r="F23" s="267" t="inlineStr">
         <is>
-          <t>Wilson Yamada</t>
+          <t>Cézar Hiraki Velázquez</t>
         </is>
       </c>
       <c r="G23" s="268" t="n"/>
@@ -18990,32 +18994,32 @@
     <row r="24">
       <c r="A24" s="267" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="B24" s="267" t="inlineStr">
         <is>
+          <t>Lucas Batista</t>
+        </is>
+      </c>
+      <c r="C24" s="267" t="inlineStr">
+        <is>
+          <t>AASP — CNJ Integração</t>
+        </is>
+      </c>
+      <c r="D24" s="267" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="E24" s="267" t="inlineStr">
+        <is>
+          <t>Desenvolvedor</t>
+        </is>
+      </c>
+      <c r="F24" s="267" t="inlineStr">
+        <is>
           <t>Cézar Hiraki Velázquez</t>
-        </is>
-      </c>
-      <c r="C24" s="267" t="inlineStr">
-        <is>
-          <t>AASP — CNJ Integração</t>
-        </is>
-      </c>
-      <c r="D24" s="267" t="inlineStr">
-        <is>
-          <t>Tech Lead / DevOps / Arquiteto</t>
-        </is>
-      </c>
-      <c r="E24" s="267" t="inlineStr">
-        <is>
-          <t>Arquiteto de Software</t>
-        </is>
-      </c>
-      <c r="F24" s="267" t="inlineStr">
-        <is>
-          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G24" s="268" t="n"/>
@@ -19031,7 +19035,7 @@
       </c>
       <c r="B25" s="267" t="inlineStr">
         <is>
-          <t>Raony Chagas</t>
+          <t>Caroline Sousa</t>
         </is>
       </c>
       <c r="C25" s="267" t="inlineStr">
@@ -19041,17 +19045,17 @@
       </c>
       <c r="D25" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior (Principal)</t>
+          <t>Analista de QA</t>
         </is>
       </c>
       <c r="E25" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor Sênior</t>
+          <t>Analista de QA</t>
         </is>
       </c>
       <c r="F25" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G25" s="268" t="n"/>
@@ -19067,7 +19071,7 @@
       </c>
       <c r="B26" s="267" t="inlineStr">
         <is>
-          <t>Mateus Veloso</t>
+          <t>Jonathan Barbosa</t>
         </is>
       </c>
       <c r="C26" s="267" t="inlineStr">
@@ -19077,17 +19081,17 @@
       </c>
       <c r="D26" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Auditor GQA (independente)</t>
         </is>
       </c>
       <c r="E26" s="267" t="inlineStr">
         <is>
-          <t>Desenvolvedor</t>
+          <t>Analista de Qualidade</t>
         </is>
       </c>
       <c r="F26" s="267" t="inlineStr">
         <is>
-          <t>Cézar Hiraki Velázquez</t>
+          <t>Abraão Oliveira</t>
         </is>
       </c>
       <c r="G26" s="268" t="n"/>
@@ -19096,108 +19100,36 @@
       <c r="J26" s="268" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="267" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="B27" s="267" t="inlineStr">
-        <is>
-          <t>Lucas Batista</t>
-        </is>
-      </c>
-      <c r="C27" s="267" t="inlineStr">
-        <is>
-          <t>AASP — CNJ Integração</t>
-        </is>
-      </c>
-      <c r="D27" s="267" t="inlineStr">
-        <is>
-          <t>Desenvolvedor</t>
-        </is>
-      </c>
-      <c r="E27" s="267" t="inlineStr">
-        <is>
-          <t>Desenvolvedor</t>
-        </is>
-      </c>
-      <c r="F27" s="267" t="inlineStr">
-        <is>
-          <t>Cézar Hiraki Velázquez</t>
-        </is>
-      </c>
+      <c r="A27" s="267" t="n"/>
+      <c r="B27" s="267" t="n"/>
+      <c r="C27" s="267" t="n"/>
+      <c r="D27" s="267" t="n"/>
+      <c r="E27" s="267" t="n"/>
+      <c r="F27" s="267" t="n"/>
       <c r="G27" s="268" t="n"/>
       <c r="H27" s="268" t="n"/>
       <c r="I27" s="109" t="n"/>
       <c r="J27" s="268" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="267" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="B28" s="267" t="inlineStr">
-        <is>
-          <t>Caroline Sousa</t>
-        </is>
-      </c>
-      <c r="C28" s="267" t="inlineStr">
-        <is>
-          <t>AASP — CNJ Integração</t>
-        </is>
-      </c>
-      <c r="D28" s="267" t="inlineStr">
-        <is>
-          <t>Analista de QA</t>
-        </is>
-      </c>
-      <c r="E28" s="267" t="inlineStr">
-        <is>
-          <t>Analista de QA</t>
-        </is>
-      </c>
-      <c r="F28" s="267" t="inlineStr">
-        <is>
-          <t>Abraão Oliveira</t>
-        </is>
-      </c>
+      <c r="A28" s="267" t="n"/>
+      <c r="B28" s="267" t="n"/>
+      <c r="C28" s="267" t="n"/>
+      <c r="D28" s="267" t="n"/>
+      <c r="E28" s="267" t="n"/>
+      <c r="F28" s="267" t="n"/>
       <c r="G28" s="268" t="n"/>
       <c r="H28" s="268" t="n"/>
       <c r="I28" s="109" t="n"/>
       <c r="J28" s="268" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="267" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="B29" s="267" t="inlineStr">
-        <is>
-          <t>Jonathan Barbosa</t>
-        </is>
-      </c>
-      <c r="C29" s="267" t="inlineStr">
-        <is>
-          <t>AASP — CNJ Integração</t>
-        </is>
-      </c>
-      <c r="D29" s="267" t="inlineStr">
-        <is>
-          <t>Auditor GQA (independente)</t>
-        </is>
-      </c>
-      <c r="E29" s="267" t="inlineStr">
-        <is>
-          <t>Analista de Qualidade</t>
-        </is>
-      </c>
-      <c r="F29" s="267" t="inlineStr">
-        <is>
-          <t>Abraão Oliveira</t>
-        </is>
-      </c>
+      <c r="A29" s="267" t="n"/>
+      <c r="B29" s="267" t="n"/>
+      <c r="C29" s="267" t="n"/>
+      <c r="D29" s="267" t="n"/>
+      <c r="E29" s="267" t="n"/>
+      <c r="F29" s="267" t="n"/>
       <c r="G29" s="268" t="n"/>
       <c r="H29" s="268" t="n"/>
       <c r="I29" s="109" t="n"/>
@@ -19302,10 +19234,10 @@
     <row r="38">
       <c r="A38" s="267" t="n"/>
       <c r="B38" s="267" t="n"/>
-      <c r="C38" s="267" t="n"/>
-      <c r="D38" s="267" t="n"/>
-      <c r="E38" s="267" t="n"/>
-      <c r="F38" s="267" t="n"/>
+      <c r="C38" s="272" t="n"/>
+      <c r="D38" s="118" t="n"/>
+      <c r="E38" s="118" t="n"/>
+      <c r="F38" s="118" t="n"/>
       <c r="G38" s="268" t="n"/>
       <c r="H38" s="268" t="n"/>
       <c r="I38" s="109" t="n"/>
@@ -19314,10 +19246,10 @@
     <row r="39">
       <c r="A39" s="267" t="n"/>
       <c r="B39" s="267" t="n"/>
-      <c r="C39" s="267" t="n"/>
-      <c r="D39" s="267" t="n"/>
-      <c r="E39" s="267" t="n"/>
-      <c r="F39" s="267" t="n"/>
+      <c r="C39" s="272" t="n"/>
+      <c r="D39" s="118" t="n"/>
+      <c r="E39" s="118" t="n"/>
+      <c r="F39" s="118" t="n"/>
       <c r="G39" s="268" t="n"/>
       <c r="H39" s="268" t="n"/>
       <c r="I39" s="109" t="n"/>
@@ -19326,10 +19258,10 @@
     <row r="40">
       <c r="A40" s="267" t="n"/>
       <c r="B40" s="267" t="n"/>
-      <c r="C40" s="267" t="n"/>
-      <c r="D40" s="267" t="n"/>
-      <c r="E40" s="267" t="n"/>
-      <c r="F40" s="267" t="n"/>
+      <c r="C40" s="272" t="n"/>
+      <c r="D40" s="118" t="n"/>
+      <c r="E40" s="118" t="n"/>
+      <c r="F40" s="118" t="n"/>
       <c r="G40" s="268" t="n"/>
       <c r="H40" s="268" t="n"/>
       <c r="I40" s="109" t="n"/>
@@ -19434,10 +19366,10 @@
     <row r="49">
       <c r="A49" s="267" t="n"/>
       <c r="B49" s="267" t="n"/>
-      <c r="C49" s="272" t="n"/>
-      <c r="D49" s="118" t="n"/>
-      <c r="E49" s="118" t="n"/>
-      <c r="F49" s="118" t="n"/>
+      <c r="C49" s="267" t="n"/>
+      <c r="D49" s="267" t="n"/>
+      <c r="E49" s="267" t="n"/>
+      <c r="F49" s="267" t="n"/>
       <c r="G49" s="268" t="n"/>
       <c r="H49" s="268" t="n"/>
       <c r="I49" s="109" t="n"/>
@@ -19446,10 +19378,10 @@
     <row r="50">
       <c r="A50" s="267" t="n"/>
       <c r="B50" s="267" t="n"/>
-      <c r="C50" s="272" t="n"/>
-      <c r="D50" s="118" t="n"/>
-      <c r="E50" s="118" t="n"/>
-      <c r="F50" s="118" t="n"/>
+      <c r="C50" s="267" t="n"/>
+      <c r="D50" s="267" t="n"/>
+      <c r="E50" s="267" t="n"/>
+      <c r="F50" s="267" t="n"/>
       <c r="G50" s="268" t="n"/>
       <c r="H50" s="268" t="n"/>
       <c r="I50" s="109" t="n"/>
@@ -19458,10 +19390,10 @@
     <row r="51">
       <c r="A51" s="267" t="n"/>
       <c r="B51" s="267" t="n"/>
-      <c r="C51" s="272" t="n"/>
-      <c r="D51" s="118" t="n"/>
-      <c r="E51" s="118" t="n"/>
-      <c r="F51" s="118" t="n"/>
+      <c r="C51" s="267" t="n"/>
+      <c r="D51" s="267" t="n"/>
+      <c r="E51" s="267" t="n"/>
+      <c r="F51" s="267" t="n"/>
       <c r="G51" s="268" t="n"/>
       <c r="H51" s="268" t="n"/>
       <c r="I51" s="109" t="n"/>
@@ -24818,42 +24750,6 @@
       <c r="H497" s="268" t="n"/>
       <c r="I497" s="109" t="n"/>
       <c r="J497" s="268" t="n"/>
-    </row>
-    <row r="498">
-      <c r="A498" s="267" t="n"/>
-      <c r="B498" s="267" t="n"/>
-      <c r="C498" s="267" t="n"/>
-      <c r="D498" s="267" t="n"/>
-      <c r="E498" s="267" t="n"/>
-      <c r="F498" s="267" t="n"/>
-      <c r="G498" s="268" t="n"/>
-      <c r="H498" s="268" t="n"/>
-      <c r="I498" s="109" t="n"/>
-      <c r="J498" s="268" t="n"/>
-    </row>
-    <row r="499">
-      <c r="A499" s="267" t="n"/>
-      <c r="B499" s="267" t="n"/>
-      <c r="C499" s="267" t="n"/>
-      <c r="D499" s="267" t="n"/>
-      <c r="E499" s="267" t="n"/>
-      <c r="F499" s="267" t="n"/>
-      <c r="G499" s="268" t="n"/>
-      <c r="H499" s="268" t="n"/>
-      <c r="I499" s="109" t="n"/>
-      <c r="J499" s="268" t="n"/>
-    </row>
-    <row r="500">
-      <c r="A500" s="267" t="n"/>
-      <c r="B500" s="267" t="n"/>
-      <c r="C500" s="267" t="n"/>
-      <c r="D500" s="267" t="n"/>
-      <c r="E500" s="267" t="n"/>
-      <c r="F500" s="267" t="n"/>
-      <c r="G500" s="268" t="n"/>
-      <c r="H500" s="268" t="n"/>
-      <c r="I500" s="109" t="n"/>
-      <c r="J500" s="268" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$3:$F$500"/>

</xml_diff>